<commit_message>
make UI polished for quiz showcase
</commit_message>
<xml_diff>
--- a/uploads/mcq-questions.xlsx
+++ b/uploads/mcq-questions.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:Y7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -445,6 +445,36 @@
       <c r="O1" t="str">
         <v>board_year</v>
       </c>
+      <c r="P1" t="str">
+        <v>combo_option_1</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>combo_option_2</v>
+      </c>
+      <c r="R1" t="str">
+        <v>combo_option_3</v>
+      </c>
+      <c r="S1" t="str">
+        <v>combo_option_4</v>
+      </c>
+      <c r="T1" t="str">
+        <v>question2</v>
+      </c>
+      <c r="U1" t="str">
+        <v>q2_option_a</v>
+      </c>
+      <c r="V1" t="str">
+        <v>q2_option_b</v>
+      </c>
+      <c r="W1" t="str">
+        <v>q2_option_c</v>
+      </c>
+      <c r="X1" t="str">
+        <v>q2_option_d</v>
+      </c>
+      <c r="Y1" t="str">
+        <v>q2_answer</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -578,9 +608,183 @@
         <v>2021</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>2</v>
+      </c>
+      <c r="B5" t="str">
+        <v>মাঠ ফসলের বৈশিষ্ট্য কোনটি?</v>
+      </c>
+      <c r="C5" t="str">
+        <v>সমস্ত ফসলকে একত্রে পরিচর্যা করা যায়</v>
+      </c>
+      <c r="D5" t="str">
+        <v>ফসলের নিবিড় পরিচর্যার প্রয়োজন হয়</v>
+      </c>
+      <c r="E5" t="str">
+        <v>নিচু ও মাঝারি জমিতে চাষ করা যায়</v>
+      </c>
+      <c r="G5" t="str">
+        <v>1</v>
+      </c>
+      <c r="H5" t="str">
+        <v>1st</v>
+      </c>
+      <c r="I5" t="str">
+        <v>Chapter 1</v>
+      </c>
+      <c r="J5" t="str">
+        <v>মাঠ ফসল</v>
+      </c>
+      <c r="K5" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="L5" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="M5" t="str">
+        <v>mcq_1780516790881</v>
+      </c>
+      <c r="O5" t="str">
+        <v/>
+      </c>
+      <c r="P5" t="str">
+        <v>i</v>
+      </c>
+      <c r="Q5" t="str">
+        <v>i, iii</v>
+      </c>
+      <c r="R5" t="str">
+        <v>ii, iii</v>
+      </c>
+      <c r="S5" t="str">
+        <v>i, ii ও iii</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>3</v>
+      </c>
+      <c r="B6" t="str">
+        <v>আসার সংরক্ষণ করার পদ্ধতি কোনটি?</v>
+      </c>
+      <c r="C6" t="str">
+        <v>দীর্ঘকালীন</v>
+      </c>
+      <c r="D6" t="str">
+        <v xml:space="preserve">স্বল্পকালীন </v>
+      </c>
+      <c r="E6" t="str">
+        <v xml:space="preserve">স্থায়ী </v>
+      </c>
+      <c r="F6" t="str">
+        <v>ডিপফ্রিজিং</v>
+      </c>
+      <c r="G6" t="str">
+        <v>B</v>
+      </c>
+      <c r="H6" t="str">
+        <v>1st</v>
+      </c>
+      <c r="I6" t="str">
+        <v>Chapter 1</v>
+      </c>
+      <c r="J6" t="str">
+        <v>মাঠ ফসল</v>
+      </c>
+      <c r="K6" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="L6" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="M6" t="str">
+        <v>mcq_1780516879169</v>
+      </c>
+      <c r="N6" t="str">
+        <v>আশা সকালে রান্নার পর দেখলো তার অনেক সবজি রয়ে গেছে। সে অবশিষ্ট সবজিগুলো পরের দিনের জন্য সংরক্ষণ করলো ।</v>
+      </c>
+      <c r="O6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>4</v>
+      </c>
+      <c r="B7" t="str">
+        <v xml:space="preserve">রবিউলের মাটি সংশোধনের প্রয়োজনীয় পদক্ষেপ হলো-  </v>
+      </c>
+      <c r="C7" t="str">
+        <v xml:space="preserve">চুন ব্যবহার করা </v>
+      </c>
+      <c r="D7" t="str">
+        <v xml:space="preserve">কাঠের ছাই প্রয়োগ করা </v>
+      </c>
+      <c r="E7" t="str">
+        <v xml:space="preserve">ট্রাইকোডার্মা ব্যবহার করা </v>
+      </c>
+      <c r="G7" t="str">
+        <v>4</v>
+      </c>
+      <c r="H7" t="str">
+        <v>1st</v>
+      </c>
+      <c r="I7" t="str">
+        <v>Chapter 1</v>
+      </c>
+      <c r="J7" t="str">
+        <v>মাঠ ফসল</v>
+      </c>
+      <c r="K7" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="L7" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="M7" t="str">
+        <v>mcq_1780518392485</v>
+      </c>
+      <c r="N7" t="str">
+        <v>রবিউল ফসলের আশানুরূপ ফলন না পেয়ে কৃষি কর্মকর্তার পরামর্শে তার জমির মাটি পরীক্ষা করে দেখলেন যে মাটির অম্লমান 4.5। পরবর্তীতে কৃষি কর্মকর্তার পরামর্শ অনুযায়ী প্রয়োজনীয় পদক্ষেপ গ্রহণ করে সুফল পান।</v>
+      </c>
+      <c r="O7" t="str">
+        <v>2021</v>
+      </c>
+      <c r="P7" t="str">
+        <v>i, ii</v>
+      </c>
+      <c r="Q7" t="str">
+        <v>i, iii</v>
+      </c>
+      <c r="R7" t="str">
+        <v>ii, iii</v>
+      </c>
+      <c r="S7" t="str">
+        <v>i, ii ও iii</v>
+      </c>
+      <c r="T7" t="str">
+        <v xml:space="preserve">রবিউলের জমির মাটি কি ধরনের? </v>
+      </c>
+      <c r="U7" t="str">
+        <v xml:space="preserve">অম্লীয় </v>
+      </c>
+      <c r="V7" t="str">
+        <v xml:space="preserve">নিরপেক্ষ </v>
+      </c>
+      <c r="W7" t="str">
+        <v xml:space="preserve">ক্ষারীয় </v>
+      </c>
+      <c r="X7" t="str">
+        <v xml:space="preserve">লবণাক্ত </v>
+      </c>
+      <c r="Y7" t="str">
+        <v>A</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Y7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>